<commit_message>
Add batch 3 products to Excel (20 SKUs)
Agrega 20 productos del lote 3 a ESTRUCTURA_RAPPI_2909206.xlsx (filas 57-76):
H23052, EMS21R, ORG3135, JBL0315, AKZR21, SD017G, KK2803, JP9063V,
H8520V, H8520R, B003MK1, H8520, SD018, JP9063L, DS152, K166B,
HD4274, K166, M6132R, B1029V

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bWxU7GBEhMMMrCBgBXSaR
</commit_message>
<xml_diff>
--- a/PRODUCTOS_RAPPI/ESTRUCTURA_RAPPI_2909206.xlsx
+++ b/PRODUCTOS_RAPPI/ESTRUCTURA_RAPPI_2909206.xlsx
@@ -676,7 +676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J56"/>
+  <dimension ref="A1:J76"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="58.7109375" customWidth="1" style="25" min="1" max="1"/>
@@ -2563,6 +2563,506 @@
       </c>
       <c r="E56" s="29" t="n">
         <v>35000</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>CORTADOR PICADOR REBANADOR PAPAS VEGETALES ACERO INOXIDABLE MD808 H23052</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>H23052</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>- – Cortadora de papas bastón – Aparato muy útil para ayudarte a preparar la comida de los más pequeños – Cuenta con dos tamaños de navajas para poder hacer papas de 10 y 12 mm de grosor – Puede cortar verduras de hasta 7cm x 7cm – Cuenta con una ven
+- Incluye garantía del fabricante
+- Envío rápido a toda Colombia
+- Producto de alta calidad
+- Ideal como regalo o para uso personal</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="n">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>PARLANTE BLUETOOTH PORTÁTIL MINI X16 ALTAVOZ INALÁMBRICO PEQUEÑO PARA MÚSICA HOGAR VIAJE ROJO EMS21R</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>EMS21R</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>- El Parlante Portátil Bluetooth Mini X16 es un altavoz compacto y versátil diseñado para disfrutar de música tanto en interiores como en exteriores
+- Cuenta con una potencia de salida de 5 W RMS mediante un altavoz de 3 pulgadas, ofreciendo un formato práctico para acompañarte en diferentes momentos
+- Su diseño cúbico y liviano incorpora una correa o asa de goma naranja en la parte superior, que facilita su transporte y también funciona como soporte ranurado para colocar un teléfono celular
+- Su conectividad permite reproducir música de forma inalámbrica mediante Bluetooth , además de ofrecer diferentes opciones de reproducción directa gracias a su puerto USB para memorias flash y ranura para tarjetas MicroSD (TF)
+- También incorpora Radio FM , interruptor deslizable de encendido y apagado y un puerto de carga mediante USB</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="n">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>JOYERO ORGANIZADOR JOYAS ACRILICO CAJONES 3 NIVELES ORG3135</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>ORG3135</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>- Organiza tus joyas con estilo y elegancia
+- Este Joyero de 3 Niveles en Acrílico es perfecto para mantener tus accesorios bien guardados y visibles
+- Con su diseño moderno y transparente, te permite encontrar rápidamente tus piezas favoritas sin complicaciones
+- Especificaciones: - Material: Acrílico de alta calidad - Niveles: 3 niveles deslizables con compartimentos ajustables - Tamaño: 23,5cm largo x 10,4cm alto x 13,5cm ancho
+- Incluye garantía del fabricante</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="n">
+        <v>42000</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>JUEGO CONDIMENTEROS X5 FRASCOS VIDRIO ACEITEROS 400ML 200ML ORGANIZADOR ESPECIAS COCINA ELEGANTE MODERNO JBL0315</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>JBL0315</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>- Capacidad: 400ml; 200ml*4 Set de Frascos Condimenteros y Aceiteros de vidrio
+- Diseño elegante y moderno
+- Vidrio resistente de alta calidad
+- Fácil de usar y limpiar
+- Incluye garantía del fabricante</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="n">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>AUDIFONOS BLUETOOTH 5.4 INALAMBRICOS DIADEMA CUELLO PANTALLA LED MICROFONO REDUCCION RUIDO WIFI PARA DEPORTES VIDEOJUEGOSS AKZR21</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>AKZR21</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>- Disfruta de una conexión rápida y estable con estos auriculares inalámbricos con Bluetooth 5
+- 4, ideales para escuchar música, realizar llamadas y disfrutar de juegos
+- Su tecnología ofrece un mayor alcance y baja latencia para una experiencia de uso más fluida y sin interrupciones
+- Su diseño con banda para el cuello proporciona una sujeción segura y cómoda durante actividades diarias o deportivas, evitando que los auriculares se caigan con el movimiento
+- Además, incorporan una pantalla LED que permite consultar fácilmente el estado de la batería, la conexión y el modo de reproducción</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="n">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>LAMPARA MESA VELADOR LUZ LED DECORATIVA RECARGABLE TACTIL 3 TONOS BATERIA 1800MAH DORMITORIO OFICINA DORADO SD017G</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>SD017G</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>- Material: Aluminio + Acrílico (pantalla)
+- El velador retro con estilo minimalista es la opción perfecta para darle un toque moderno a cualquier espacio! Cuenta con selector de 3 colores de iluminación: (Luz blanca, luz neutra y luz cálida) que le permite cambiar fácilmente el brillo presio
+- Tanto el encendido y apagado, como el cambio de intensidad y color de la luz se realiza de forma táctil, presionando la parte superior de la lámpara
+- Para cambiar la intensidad de la luz se debe mantener presionado el sensor táctil
+- Tiempo de duración de la batería prolongada: batería integrada de 1800 mAh, con una autonomía de 12 hs apróximadamente</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="n">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>RELOJ DIGITAL PARED NUMEROS GRANDES CALENDARIO TEMPERATURA ALARMA KK-2803</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>KK2803</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>- Reloj Digital De Pared Numero Grande Calendario Temperatura Organiza tu tiempo con estilo
+- Este reloj digital es ideal para tu hogar u oficina
+- Con números grandes y claros, permite ver la hora fácilmente, incluso a distancia
+- Su diseño sobrio y minimalista combina con cualquier tipo de decoración, ya sea colocado en la pared o sobre una superficie
+- Este modelo incluye: Alarma: para mantener tus citas y compromisos bajo control</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="n">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>BOLSO VIAJE FASHION DEPORTIVO IMPERMEABLE GRANDE COMPARTIMENTO HÚMEDO SECO CORREA DESMONTABLE GIMNASIO EQUIPAJE MULTIUSOS VINOTINTO JP9063V</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>JP9063V</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>- Diseño lujoso: esta bolsa de lona de gran tamaño cuenta con una construcción elegante y duradera, perfecta para aventuras de viaje y sesiones de gimnasio
+- Compartimento impermeable: cuenta con un compartimento impermeable dedicado para mantener sus elementos esenciales secos y protegidos
+- Transporte multifuncional: opciones de transporte versátiles que incluyen asas superiores y una correa de hombro desmontable para un transporte cómodo
+- Separación seca y húmeda: compartimentos separados le permiten organizar cuidadosamente los artículos secos y húmedos
+- Prácticos bolsillos laterales: bolsillos laterales convenientemente colocados que proporcionan un fácil acceso a objetos más pequeños</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>LAMPARA CAPERUZA PARA CAMPING VERDE PORTATIL DE EXTERIOR ILUMINACION PARA ACAMPAR SENDERISMO Y VIAJE K20 H8520V</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>H8520V</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>- En la parte superior cuenta con un gancho metalico
+- Esto le da mayor versatilidad en el uso, ya que te permitira usarla no solo apoyandola en una superficie sino tambien colgarla tanto del techo de una carpa o de la rama de un arbol como se observa en las imagenes
+- Es tambien un elemento decorativo agradable debido a su diseño retro
+- Tiene un ángulo de haz de luz de 360 grados altamente brillante, que puede proporcionar suficiente brillo
+- Se enciende girando la perilla y ademas es dimerizable, por lo que vas a poder regular la intensidad de la luz</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>LAMPARA CAPERUZA PARA CAMPING ROJA PORTATIL DE EXTERIOR ILUMINACION PARA ACAMPAR SENDERISMO Y VIAJE ROJO K20 H8520R</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>H8520R</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>- En la parte superior cuenta con un gancho metalico
+- Esto le da mayor versatilidad en el uso, ya que te permitira usarla no solo apoyandola en una superficie sino tambien colgarla tanto del techo de una carpa o de la rama de un arbol como se observa en las imagenes
+- Es tambien un elemento decorativo agradable debido a su diseño retro
+- Tiene un ángulo de haz de luz de 360 grados altamente brillante, que puede proporcionar suficiente brillo
+- Se enciende girando la perilla y ademas es dimerizable, por lo que vas a poder regular la intensidad de la luz</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>SOPORTE DE COCINA PARA CUBIERTOS CON AFILADOR DE CUCHILLOS VERDE TPL B003MK1</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>B003MK1</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>-Materiales ABS seleccionados de alta calidad, diseño grueso, buena capacidad de carga
+- Hermoso y elegante, lleno de textura, no se deforma fácilmente, y se puede utilizar durante mucho tiempo
+-El estante de drenaje para palillos está equipado con orificios de drenaje y una base para facilitar el drenaje y no mojar la mesa
+- Los pies de goma en la base del estante de almacenamiento son antideslizantes y suaves para evitar arañazos en la encimera y la estabilidad de la base ancha
+-Afilador de cuchillos + estante de herramientas + cesta de cuchillos multifunción, diseño compacto, peso ligero, ahorra espacio en la mesa</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="n">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>LAMPARA CAPERUZA PARA CAMPING NEGRA PORTATIL DE EXTERIOR ILUMINACION PARA ACAMPAR SENDERISMO Y VIAJE K20 H8520</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>H8520</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>- En la parte superior cuenta con un gancho metalico
+- Esto le da mayor versatilidad en el uso, ya que te permitira usarla no solo apoyandola en una superficie sino tambien colgarla tanto del techo de una carpa o de la rama de un arbol como se observa en las imagenes
+- Es tambien un elemento decorativo agradable debido a su diseño retro
+- Tiene un ángulo de haz de luz de 360 grados altamente brillante, que puede proporcionar suficiente brillo
+- Se enciende girando la perilla y ademas es dimerizable, por lo que vas a poder regular la intensidad de la luz</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>LAMPARA MESA LED DECORATIVO RECARGABLE INALAMBRICO TACTIL 3 TONOS LUZ METAL ACRILICO MODERNO PLATEADO SD018</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>SD018</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>- SIMPLE MODERNO: con un diseño industrial minimalista, la luz LED se puede colocar en cualquier lugar, como una mesita de noche, una estantería, una mesa, una mesa de comedor, etc
+- INALÁMBRICO Y RECARGABLE: la lámpara de mesa inalámbrica tiene una batería recargable de 1800 mAh incorporada
+- 3 COLORES: esta lámpara de mesa tiene 3 colores de iluminación: luz blanca, blanca cálida, luz , puede seleccionar usar según las necesidades, presione prolongadamente para atenuación continua
+- La lámpara de mesa adopta una carcasa de metal, una pantalla de acrílico transparente, un proceso de galvanoplastia superficial y un diseño de base antideslizante, resistente y estable
+- Diseño elegante: construido con una carcasa de metal resistente y una pantalla acrílica transparente, esta lámpara combina durabilidad con elegancia</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="n">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>BOLSO VIAJE FASHION DEPORTIVO IMPERMEABLE GRANDE COMPARTIMENTO HÚMEDO SECO CORREA DESMONTABLE GIMNASIO EQUIPAJE MULTIUSOS LILA JP9063L</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>JP9063L</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>- Diseño lujoso: esta bolsa de lona de gran tamaño cuenta con una construcción elegante y duradera, perfecta para aventuras de viaje y sesiones de gimnasio
+- Compartimento impermeable: cuenta con un compartimento impermeable dedicado para mantener sus elementos esenciales secos y protegidos
+- Transporte multifuncional: opciones de transporte versátiles que incluyen asas superiores y una correa de hombro desmontable para un transporte cómodo
+- Separación seca y húmeda: compartimentos separados le permiten organizar cuidadosamente los artículos secos y húmedos
+- Prácticos bolsillos laterales: bolsillos laterales convenientemente colocados que proporcionan un fácil acceso a objetos más pequeños</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>ARENA SINTÉTICA MÁGICA INFANTIL SENSORIAL CREATIVA JUEGO DE CONSTRUCCIÓN COORDINACIÓN MANO OJO DS152</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>DS152</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>- ¡Descubre la Magia de la Arena Mágica! Transforma el tiempo de juego de tus hijos con Magic Sand, un juguete que no solo divierte, sino que también estimula la imaginación y la creatividad
+- Ideal para mejorar la coordinación mano-ojo, este producto es perfecto para mantener a los más pequeños ocupados y motivados
+- Características Destacadas: • Versatilidad: Perfecto para usar en el patio trasero, playa, piscina o interior
+- Sensory Sand ofrece un diseño único que permite a los niños explorar la vida marina y áreas de construcción mientras juegan
+- • Materiales de Alta Calidad: Fabricado en ABS duradero, este juguete es seguro, resistente al desgaste y suave al tacto, garantizando horas de diversión sin preocupaciones</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="n">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>TERMO VASO TÉRMICO DIGITAL ACERO INOXIDABLE PANTALLA LED TEMPERATURA TAPA HERMÉTICA FRÍO CALIENTE PORTÁTIL BEIGE K166B</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>K166B</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>- Este Termo Vaso Térmico con pantalla digital es el compañero ideal para tus días activos
+- Su diseño moderno y funcional te permite mantener tus bebidas calientes o frías por más tiempo, mientras su pantalla LED en la tapa te muestra en segundos la temperatura exacta del líquido interior
+- Es perfecto para llevar café, té, agua o cualquier bebida favorita a la oficina, al gimnasio o de viaje
+- Fabricado con materiales resistentes y de alta calidad, este termo combina elegancia con practicidad
+- Su tapa hermética evita derrames, y su tamaño es ideal para bolsos o portavasos de auto</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="n">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>XIAOMI IN-EAR HEADPHONES BASIC SILVER 14274 AUDÍFONOS ALÁMBRICOS MICRÓFONO CONTROL CABLE ANTIENTREDOS HD4274</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>HD4274</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>- Su diseño ergonómico y ultraligero te brinda comodidad durante horas de uso
+- Fabricados con materiales de alta calidad, estos audífonos ofrecen una experiencia auditiva excepcional, con bajos profundos y agudos claros, optimizados para diversos géneros musicales como pop, rock y dance
+- Su cable plano, resistente a enredos, incorpora una envoltura interior de Kevlar para una mayor durabilidad, mientras que el sistema de amortiguación de tercera generación garantiza un sonido balanceado y transparente
+- Contesta llamadas y controla tu música con un solo botón, compatible con dispositivos Android e iOS
+- Incluye garantía del fabricante</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="n">
+        <v>32000</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>TERMO VASO TÉRMICO DIGITAL ACERO INOXIDABLE PANTALLA LED TEMPERATURA TAPA HERMÉTICA FRÍO CALIENTE PORTÁTIL NEGRO K166</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>K166</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>- Este Termo Vaso Térmico con pantalla digital es el compañero ideal para tus días activos
+- Su diseño moderno y funcional te permite mantener tus bebidas calientes o frías por más tiempo, mientras su pantalla LED en la tapa te muestra en segundos la temperatura exacta del líquido interior
+- Es perfecto para llevar café, té, agua o cualquier bebida favorita a la oficina, al gimnasio o de viaje
+- Fabricado con materiales resistentes y de alta calidad, este termo combina elegancia con practicidad
+- Su tapa hermética evita derrames, y su tamaño es ideal para bolsos o portavasos de auto</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="n">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>MORRAL VIAJE DEPORTIVO IMPERMEABLE HONGFU BOLSO GIMNASIO GRAN CAPACIDAD PLEGABLE MULTIUSOS 20741 ROSADO M6132R</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>M6132R</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>- La bolsa de viaje está hecha con tela ligera impermeable y Oxford, sólida, antiarrugas, resistente al desgaste, impermeable, fácil de fregar y duradera
+- Puede ayudarte a separar artículos secos y húmedos
+- Si tienes ropa mojada, toallas y artículos de tocador, puedes ponerlos en esta bolsa
+- Te hace sentir más cómodo en tu entrenamiento diario y viaje
+- Adecuado para entrenamientos, viajes, actividades deportivas, tenis, baloncesto, yoga, pesca, caza, camping, senderismo y muchas actividades al aire libre</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>CONJUNTO DE LICRA DEPORTIVO MUJER GYM YOGA SUJETADOR DEPORTIVO LEGGINGS CINTURA ALTA SIN COSTURAS S-M VERDE B1029V</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>B1029V</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>- Cómodo y elástico: el nailon proporciona un alto agarre y absorción del sudor
+- El elastano proporciona estiramiento adicional para un mejor ajuste
+- Trajes deportivos: los conjuntos de yoga incluyen un sujetador deportivo y leggings de cintura alta
+- conjunto deportivo mujer ropa deportiva mujer conjunto gym conjunto gimnasio mujer ropa gym mujer conjunto deporte mujer sujetador deportivo mujer conjunto fitness mujer mallas gimnasio mujer deportivas mujer gym
+- Diseño sin costuras: material elástico en cuatro direcciones, suave y compresible, transpirable y absorbe la humedad, los trajes de yoga se adaptan perfectamente a tu cuerpo y protegen tu pecho de la presión</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="n">
+        <v>40000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fill categories for batch 3 products in Excel
Asigna categorías Rappi a los 20 productos del lote 3 (filas 57-76)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bWxU7GBEhMMMrCBgBXSaR
</commit_message>
<xml_diff>
--- a/PRODUCTOS_RAPPI/ESTRUCTURA_RAPPI_2909206.xlsx
+++ b/PRODUCTOS_RAPPI/ESTRUCTURA_RAPPI_2909206.xlsx
@@ -2585,7 +2585,11 @@
 - Ideal como regalo o para uso personal</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr"/>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Cuidado y limpieza del hogar</t>
+        </is>
+      </c>
       <c r="E57" t="n">
         <v>45000</v>
       </c>
@@ -2610,7 +2614,11 @@
 - También incorpora Radio FM , interruptor deslizable de encendido y apagado y un puerto de carga mediante USB</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr"/>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Tecnología</t>
+        </is>
+      </c>
       <c r="E58" t="n">
         <v>45000</v>
       </c>
@@ -2635,7 +2643,11 @@
 - Incluye garantía del fabricante</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr"/>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Decoración y hogar</t>
+        </is>
+      </c>
       <c r="E59" t="n">
         <v>42000</v>
       </c>
@@ -2660,7 +2672,11 @@
 - Incluye garantía del fabricante</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr"/>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Decoración y hogar</t>
+        </is>
+      </c>
       <c r="E60" t="n">
         <v>48000</v>
       </c>
@@ -2685,7 +2701,11 @@
 - Además, incorporan una pantalla LED que permite consultar fácilmente el estado de la batería, la conexión y el modo de reproducción</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Tecnología</t>
+        </is>
+      </c>
       <c r="E61" t="n">
         <v>45000</v>
       </c>
@@ -2710,7 +2730,11 @@
 - Tiempo de duración de la batería prolongada: batería integrada de 1800 mAh, con una autonomía de 12 hs apróximadamente</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr"/>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Decoración y hogar</t>
+        </is>
+      </c>
       <c r="E62" t="n">
         <v>35000</v>
       </c>
@@ -2735,7 +2759,11 @@
 - Este modelo incluye: Alarma: para mantener tus citas y compromisos bajo control</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr"/>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Decoración y hogar</t>
+        </is>
+      </c>
       <c r="E63" t="n">
         <v>45000</v>
       </c>
@@ -2760,7 +2788,11 @@
 - Prácticos bolsillos laterales: bolsillos laterales convenientemente colocados que proporcionan un fácil acceso a objetos más pequeños</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr"/>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Moda</t>
+        </is>
+      </c>
       <c r="E64" t="n">
         <v>40000</v>
       </c>
@@ -2785,7 +2817,11 @@
 - Se enciende girando la perilla y ademas es dimerizable, por lo que vas a poder regular la intensidad de la luz</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr"/>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Ferretería y jardín</t>
+        </is>
+      </c>
       <c r="E65" t="n">
         <v>40000</v>
       </c>
@@ -2810,7 +2846,11 @@
 - Se enciende girando la perilla y ademas es dimerizable, por lo que vas a poder regular la intensidad de la luz</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr"/>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Ferretería y jardín</t>
+        </is>
+      </c>
       <c r="E66" t="n">
         <v>40000</v>
       </c>
@@ -2835,7 +2875,11 @@
 -Afilador de cuchillos + estante de herramientas + cesta de cuchillos multifunción, diseño compacto, peso ligero, ahorra espacio en la mesa</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr"/>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Decoración y hogar</t>
+        </is>
+      </c>
       <c r="E67" t="n">
         <v>35000</v>
       </c>
@@ -2860,7 +2904,11 @@
 - Se enciende girando la perilla y ademas es dimerizable, por lo que vas a poder regular la intensidad de la luz</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr"/>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Ferretería y jardín</t>
+        </is>
+      </c>
       <c r="E68" t="n">
         <v>40000</v>
       </c>
@@ -2885,7 +2933,11 @@
 - Diseño elegante: construido con una carcasa de metal resistente y una pantalla acrílica transparente, esta lámpara combina durabilidad con elegancia</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr"/>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Decoración y hogar</t>
+        </is>
+      </c>
       <c r="E69" t="n">
         <v>35000</v>
       </c>
@@ -2910,7 +2962,11 @@
 - Prácticos bolsillos laterales: bolsillos laterales convenientemente colocados que proporcionan un fácil acceso a objetos más pequeños</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr"/>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Moda</t>
+        </is>
+      </c>
       <c r="E70" t="n">
         <v>40000</v>
       </c>
@@ -2935,7 +2991,11 @@
 - • Materiales de Alta Calidad: Fabricado en ABS duradero, este juguete es seguro, resistente al desgaste y suave al tacto, garantizando horas de diversión sin preocupaciones</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr"/>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Juguetería</t>
+        </is>
+      </c>
       <c r="E71" t="n">
         <v>45000</v>
       </c>
@@ -2960,7 +3020,11 @@
 - Su tapa hermética evita derrames, y su tamaño es ideal para bolsos o portavasos de auto</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr"/>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Decoración y hogar</t>
+        </is>
+      </c>
       <c r="E72" t="n">
         <v>45000</v>
       </c>
@@ -2985,7 +3049,11 @@
 - Incluye garantía del fabricante</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr"/>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Tecnología</t>
+        </is>
+      </c>
       <c r="E73" t="n">
         <v>32000</v>
       </c>
@@ -3010,7 +3078,11 @@
 - Su tapa hermética evita derrames, y su tamaño es ideal para bolsos o portavasos de auto</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr"/>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Decoración y hogar</t>
+        </is>
+      </c>
       <c r="E74" t="n">
         <v>45000</v>
       </c>
@@ -3035,7 +3107,11 @@
 - Adecuado para entrenamientos, viajes, actividades deportivas, tenis, baloncesto, yoga, pesca, caza, camping, senderismo y muchas actividades al aire libre</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr"/>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Moda</t>
+        </is>
+      </c>
       <c r="E75" t="n">
         <v>30000</v>
       </c>
@@ -3060,7 +3136,11 @@
 - Diseño sin costuras: material elástico en cuatro direcciones, suave y compresible, transpirable y absorbe la humedad, los trajes de yoga se adaptan perfectamente a tu cuerpo y protegen tu pecho de la presión</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr"/>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Deportes y fitness</t>
+        </is>
+      </c>
       <c r="E76" t="n">
         <v>40000</v>
       </c>

</xml_diff>

<commit_message>
Add batch 4 products to Excel (12 new SKUs)
Agrega 12 productos nuevos del lote 4 (filas 77-88):
BST09T, H4896, H5152A, H5152V, H5636C, H5636M, K017MK1,
M1123, M1123R, SD018G, TCP311, TCP311D

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bWxU7GBEhMMMrCBgBXSaR
</commit_message>
<xml_diff>
--- a/PRODUCTOS_RAPPI/ESTRUCTURA_RAPPI_2909206.xlsx
+++ b/PRODUCTOS_RAPPI/ESTRUCTURA_RAPPI_2909206.xlsx
@@ -676,7 +676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J76"/>
+  <dimension ref="A1:J88"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="58.7109375" customWidth="1" style="25" min="1" max="1"/>
@@ -3143,6 +3143,344 @@
       </c>
       <c r="E76" t="n">
         <v>40000</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>TECLADO BASIK TECH MULTIMEDIA USB PARA COMPUTADOR PC OFICINA TRABAJO ESTUDIO ACCESORIO DE ESCRITORIO BST09T</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>BST09T</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>- Disfruta de una experiencia cómoda y práctica con este teclado multimedia de 121 teclas, diseñado para acompañarte durante jornadas de trabajo, estudio o entretenimiento
+- Incluye 16 teclas adicionales con acceso directo a funciones como volumen, reproducción y navegación, facilitando el control de diferentes funciones desde el teclado
+- Su diseño ergonómico y resistente está pensado para ofrecer comodidad durante largas horas de uso, mientras que la distribución en español y las teclas de color permiten una experiencia versátil para jugar, estudiar o trabajar
+- Además, incorpora teclas laminadas que ayudan a resistir el desgaste por el uso frecuente
+- Cuenta con conexión USB 2.0 Plug &amp; Play, por lo que puedes conectarlo y utilizarlo sin necesidad de instalar software adicional</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Tecnología</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>CAFETERA PRENSA FRANCESA DE VIDRIO PARA CAFÉ A ÉMBOLO 1000ML 1 LITRO H4896</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>H4896</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>- Cafetera Prensa Francesa A Embolo Vidrio 1 Litro
+- Capacidad: 1000ml
+- Material: vidrio</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Cuidado y limpieza del hogar</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>MINI LICUADORA PORTÁTIL RECARGABLE USB AZUL 450ML 12 CUCHILLAS 3 VELOCIDADES PARA BATIDOS Y JUGOS HS-860 H5152A</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>H5152A</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>- Recargable por USB y portátil: con su diseño compacto y liviano y su función recargable por USB, esta licuadora portátil es ideal para disfrutar de bebidas refrescantes en casa, en la oficina o mientras viaja
+- Potente de 12 cuchillas: Con 12 cuchillas ultraafiladas y un motor de alta velocidad, esta licuadora portátil tritura fácilmente hielo y mezcla frutas en jugos o batidos suaves y ricos en nutrientes en segundos
+- Modo multifuncional de 3 velocidades: con una pantalla digital y 3 configuraciones de velocidad ajustables, este exprimidor en miniatura le permite personalizar la mezcla de una variedad de bebidas, desde batidos hasta batidos</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Cuidado y limpieza del hogar</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>MINI LICUADORA PORTÁTIL RECARGABLE USB VERDE 450ML 12 CUCHILLAS 3 VELOCIDADES PARA BATIDOS Y JUGOS HS-860 H5152V</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>H5152V</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>- Recargable por USB y portátil: con su diseño compacto y liviano y su función recargable por USB, esta licuadora portátil es ideal para disfrutar de bebidas refrescantes en casa, en la oficina o mientras viaja
+- Potente de 12 cuchillas: Con 12 cuchillas ultraafiladas y un motor de alta velocidad, esta licuadora portátil tritura fácilmente hielo y mezcla frutas en jugos o batidos suaves y ricos en nutrientes en segundos
+- Modo multifuncional de 3 velocidades: con una pantalla digital y 3 configuraciones de velocidad ajustables, este exprimidor en miniatura le permite personalizar la mezcla de una variedad de bebidas, desde batidos hasta batidos</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Cuidado y limpieza del hogar</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>FORRO PUERTA NAVIDEÑO RENO DECORACION 2M X90CM H5636C</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>H5636C</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>- Diseños variados, le puede llegar el motivo en aleatorio MEDIDAS: 2M de alto x 90cm de ancho</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Decoración y hogar</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>FUNDA FORRO DECORATIVO PARA PUERTAS NAVIDEÑO MUÑECO DE NIEVE H5636M</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>H5636M</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>- Diseños variados, le puede llegar el motivo en aleatorio
+- Estira hasta 2M de altura
+- Añadir a la puerta delantera: Llame fácilmente la atención con esta cubierta de puerta de Navidad de diseño temático de Navidad de invierno
+- Los colores vibrantes y los patrones intrincados agregarán encanto a la puerta principal de su casa
+- Adecuado para la mayoría de las puertas, es una manera perfecta de dar la bienvenida a familiares y amigos con una atractiva entrada</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Decoración y hogar</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>NIVELADOR LASER DE 3 BURBUJAS CON METRO ALINEADOR MULTRIPROPÓSITO TPL K017MK1</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>K017MK1</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>- Nivel láser fixit level pro 3: herramienta esencial para trabajos de precisión
+- Proyecta líneas horizontales y verticales para instalaciones perfectas
+- Alcance de 2.5 m ideal para interiores y espacios reducidos
+- Incorpora regla métrica y estándar para mediciones rápidas y precisas
+- 3 niveles de burbuja para una alineación impecable</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Ferretería y jardín</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>BOLSO DAMA CARTERA PORTACELULAR CUERO SUAVE TÁCTIL CORREA AJUSTABLE CREMALLERA COMPARTIMENTOS 11X18CM VERDE M1123</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>M1123</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>- Bolso Billetera de Cuero Suave para Móvil: Elegancia y Funcionalidad en tus Manos
+- Tacto Sensible y Práctico: Diseñado con una ventana transparente, este bolso para teléfono permite un fácil acceso sin necesidad de sacar el móvil
+- Su material sensible al tacto facilita el manejo del teléfono mientras permanece protegido
+- Diseño Chic y Funcional: Compacto y elegante, mide 11 x 18 x 4 cm
+- Cuenta con un cierre con cremallera y solapa magnética con botón a presión, ofreciendo un cierre seguro y fácil de usar en tu día a día</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Moda</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>37000</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>BOLSO DAMA CARTERA PORTACELULAR CUERO SUAVE TÁCTIL CORREA AJUSTABLE CREMALLERA COMPARTIMENTOS 11X18CM ROSADO M1123R</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>M1123R</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>- Bolso Billetera de Cuero Suave para Móvil: Elegancia y Funcionalidad en tus Manos
+- Tacto Sensible y Práctico: Diseñado con una ventana transparente, este bolso para teléfono permite un fácil acceso sin necesidad de sacar el móvil
+- Su material sensible al tacto facilita el manejo del teléfono mientras permanece protegido
+- Diseño Chic y Funcional: Compacto y elegante, mide 11 x 18 x 4 cm
+- Cuenta con un cierre con cremallera y solapa magnética con botón a presión, ofreciendo un cierre seguro y fácil de usar en tu día a día</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Moda</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>37000</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>LAMPARA MESA LED DECORATIVO RECARGABLE INALAMBRICO TACTIL 3 TONOS LUZ METAL ACRILICO MODERNO DORADO SD018G</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>SD018G</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>- SIMPLE MODERNO: con un diseño industrial minimalista, la luz LED se puede colocar en cualquier lugar, como una mesita de noche, una estantería, una mesa, una mesa de comedor, etc
+- INALÁMBRICO Y RECARGABLE: la lámpara de mesa inalámbrica tiene una batería recargable de 1800 mAh incorporada
+- 3 COLORES: esta lámpara de mesa tiene 3 colores de iluminación: luz blanca, blanca cálida, luz , puede seleccionar usar según las necesidades, presione prolongadamente para atenuación continua
+- La lámpara de mesa adopta una carcasa de metal, una pantalla de acrílico transparente, un proceso de galvanoplastia superficial y un diseño de base antideslizante, resistente y estable
+- Diseño elegante: construido con una carcasa de metal resistente y una pantalla acrílica transparente, esta lámpara combina durabilidad con elegancia</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Decoración y hogar</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>BANDEJA 3 NIVELES ACRÍLICO DORADO TORRE POSTRES CUPCAKES DULCES APERITIVOS DESMONTABLE ELEGANTE PLATEADO TCP311</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>TCP311</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>- Ideal para fiestas, bodas, cumpleaños, baby showers, eventos corporativos o incluso para la decoración del hogar, este soporte es perfecto para exhibir dulces gourmet, cupcakes, minitartas, frutas, aperitivos salados o pequeños obsequios
+- Su diseño sofisticado aporta un toque de lujo a la mesa, mientras que el material acrílico de alta calidad garantiza que sea ligero, duradero y fácil de limpiar
+- Gracias a su estructura robusta y acabado en tono dorado, combina a la perfección con diversos estilos de decoración, desde el clásico hasta el moderno
+- Material: Acrílico resistente
+- Color: Transparente con detalles dorados</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Decoración y hogar</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>BANDEJA 3 NIVELES ACRÍLICO DORADO TORRE POSTRES CUPCAKES DULCES APERITIVOS DESMONTABLE ELEGANTE DORADO TCP311D</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>TCP311D</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>- Ideal para fiestas, bodas, cumpleaños, baby showers, eventos corporativos o incluso para la decoración del hogar, este soporte es perfecto para exhibir dulces gourmet, cupcakes, minitartas, frutas, aperitivos salados o pequeños obsequios
+- Su diseño sofisticado aporta un toque de lujo a la mesa, mientras que el material acrílico de alta calidad garantiza que sea ligero, duradero y fácil de limpiar
+- Gracias a su estructura robusta y acabado en tono dorado, combina a la perfección con diversos estilos de decoración, desde el clásico hasta el moderno
+- Material: Acrílico resistente
+- Color: Transparente con detalles dorados</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Decoración y hogar</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>45000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Split batch 4 into its own Excel document
Mueve los 12 productos del lote 4 a un nuevo documento
ESTRUCTURA_RAPPI_LOTE4.xlsx (mismo formato) y los quita del
Excel principal ESTRUCTURA_RAPPI_2909206.xlsx, para evitar tener
que borrar filas anteriores en cada entrega.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bWxU7GBEhMMMrCBgBXSaR
</commit_message>
<xml_diff>
--- a/PRODUCTOS_RAPPI/ESTRUCTURA_RAPPI_2909206.xlsx
+++ b/PRODUCTOS_RAPPI/ESTRUCTURA_RAPPI_2909206.xlsx
@@ -676,7 +676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J88"/>
+  <dimension ref="A1:J76"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="58.7109375" customWidth="1" style="25" min="1" max="1"/>
@@ -3143,344 +3143,6 @@
       </c>
       <c r="E76" t="n">
         <v>40000</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>TECLADO BASIK TECH MULTIMEDIA USB PARA COMPUTADOR PC OFICINA TRABAJO ESTUDIO ACCESORIO DE ESCRITORIO BST09T</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>BST09T</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>- Disfruta de una experiencia cómoda y práctica con este teclado multimedia de 121 teclas, diseñado para acompañarte durante jornadas de trabajo, estudio o entretenimiento
-- Incluye 16 teclas adicionales con acceso directo a funciones como volumen, reproducción y navegación, facilitando el control de diferentes funciones desde el teclado
-- Su diseño ergonómico y resistente está pensado para ofrecer comodidad durante largas horas de uso, mientras que la distribución en español y las teclas de color permiten una experiencia versátil para jugar, estudiar o trabajar
-- Además, incorpora teclas laminadas que ayudan a resistir el desgaste por el uso frecuente
-- Cuenta con conexión USB 2.0 Plug &amp; Play, por lo que puedes conectarlo y utilizarlo sin necesidad de instalar software adicional</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>Tecnología</t>
-        </is>
-      </c>
-      <c r="E77" t="n">
-        <v>35000</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>CAFETERA PRENSA FRANCESA DE VIDRIO PARA CAFÉ A ÉMBOLO 1000ML 1 LITRO H4896</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>H4896</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>- Cafetera Prensa Francesa A Embolo Vidrio 1 Litro
-- Capacidad: 1000ml
-- Material: vidrio</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>Cuidado y limpieza del hogar</t>
-        </is>
-      </c>
-      <c r="E78" t="n">
-        <v>45000</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>MINI LICUADORA PORTÁTIL RECARGABLE USB AZUL 450ML 12 CUCHILLAS 3 VELOCIDADES PARA BATIDOS Y JUGOS HS-860 H5152A</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>H5152A</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>- Recargable por USB y portátil: con su diseño compacto y liviano y su función recargable por USB, esta licuadora portátil es ideal para disfrutar de bebidas refrescantes en casa, en la oficina o mientras viaja
-- Potente de 12 cuchillas: Con 12 cuchillas ultraafiladas y un motor de alta velocidad, esta licuadora portátil tritura fácilmente hielo y mezcla frutas en jugos o batidos suaves y ricos en nutrientes en segundos
-- Modo multifuncional de 3 velocidades: con una pantalla digital y 3 configuraciones de velocidad ajustables, este exprimidor en miniatura le permite personalizar la mezcla de una variedad de bebidas, desde batidos hasta batidos</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>Cuidado y limpieza del hogar</t>
-        </is>
-      </c>
-      <c r="E79" t="n">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>MINI LICUADORA PORTÁTIL RECARGABLE USB VERDE 450ML 12 CUCHILLAS 3 VELOCIDADES PARA BATIDOS Y JUGOS HS-860 H5152V</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>H5152V</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>- Recargable por USB y portátil: con su diseño compacto y liviano y su función recargable por USB, esta licuadora portátil es ideal para disfrutar de bebidas refrescantes en casa, en la oficina o mientras viaja
-- Potente de 12 cuchillas: Con 12 cuchillas ultraafiladas y un motor de alta velocidad, esta licuadora portátil tritura fácilmente hielo y mezcla frutas en jugos o batidos suaves y ricos en nutrientes en segundos
-- Modo multifuncional de 3 velocidades: con una pantalla digital y 3 configuraciones de velocidad ajustables, este exprimidor en miniatura le permite personalizar la mezcla de una variedad de bebidas, desde batidos hasta batidos</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>Cuidado y limpieza del hogar</t>
-        </is>
-      </c>
-      <c r="E80" t="n">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>FORRO PUERTA NAVIDEÑO RENO DECORACION 2M X90CM H5636C</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>H5636C</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>- Diseños variados, le puede llegar el motivo en aleatorio MEDIDAS: 2M de alto x 90cm de ancho</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Decoración y hogar</t>
-        </is>
-      </c>
-      <c r="E81" t="n">
-        <v>30000</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>FUNDA FORRO DECORATIVO PARA PUERTAS NAVIDEÑO MUÑECO DE NIEVE H5636M</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>H5636M</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>- Diseños variados, le puede llegar el motivo en aleatorio
-- Estira hasta 2M de altura
-- Añadir a la puerta delantera: Llame fácilmente la atención con esta cubierta de puerta de Navidad de diseño temático de Navidad de invierno
-- Los colores vibrantes y los patrones intrincados agregarán encanto a la puerta principal de su casa
-- Adecuado para la mayoría de las puertas, es una manera perfecta de dar la bienvenida a familiares y amigos con una atractiva entrada</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>Decoración y hogar</t>
-        </is>
-      </c>
-      <c r="E82" t="n">
-        <v>30000</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>NIVELADOR LASER DE 3 BURBUJAS CON METRO ALINEADOR MULTRIPROPÓSITO TPL K017MK1</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>K017MK1</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>- Nivel láser fixit level pro 3: herramienta esencial para trabajos de precisión
-- Proyecta líneas horizontales y verticales para instalaciones perfectas
-- Alcance de 2.5 m ideal para interiores y espacios reducidos
-- Incorpora regla métrica y estándar para mediciones rápidas y precisas
-- 3 niveles de burbuja para una alineación impecable</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>Ferretería y jardín</t>
-        </is>
-      </c>
-      <c r="E83" t="n">
-        <v>45000</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>BOLSO DAMA CARTERA PORTACELULAR CUERO SUAVE TÁCTIL CORREA AJUSTABLE CREMALLERA COMPARTIMENTOS 11X18CM VERDE M1123</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>M1123</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>- Bolso Billetera de Cuero Suave para Móvil: Elegancia y Funcionalidad en tus Manos
-- Tacto Sensible y Práctico: Diseñado con una ventana transparente, este bolso para teléfono permite un fácil acceso sin necesidad de sacar el móvil
-- Su material sensible al tacto facilita el manejo del teléfono mientras permanece protegido
-- Diseño Chic y Funcional: Compacto y elegante, mide 11 x 18 x 4 cm
-- Cuenta con un cierre con cremallera y solapa magnética con botón a presión, ofreciendo un cierre seguro y fácil de usar en tu día a día</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr">
-        <is>
-          <t>Moda</t>
-        </is>
-      </c>
-      <c r="E84" t="n">
-        <v>37000</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>BOLSO DAMA CARTERA PORTACELULAR CUERO SUAVE TÁCTIL CORREA AJUSTABLE CREMALLERA COMPARTIMENTOS 11X18CM ROSADO M1123R</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>M1123R</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>- Bolso Billetera de Cuero Suave para Móvil: Elegancia y Funcionalidad en tus Manos
-- Tacto Sensible y Práctico: Diseñado con una ventana transparente, este bolso para teléfono permite un fácil acceso sin necesidad de sacar el móvil
-- Su material sensible al tacto facilita el manejo del teléfono mientras permanece protegido
-- Diseño Chic y Funcional: Compacto y elegante, mide 11 x 18 x 4 cm
-- Cuenta con un cierre con cremallera y solapa magnética con botón a presión, ofreciendo un cierre seguro y fácil de usar en tu día a día</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>Moda</t>
-        </is>
-      </c>
-      <c r="E85" t="n">
-        <v>37000</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>LAMPARA MESA LED DECORATIVO RECARGABLE INALAMBRICO TACTIL 3 TONOS LUZ METAL ACRILICO MODERNO DORADO SD018G</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>SD018G</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>- SIMPLE MODERNO: con un diseño industrial minimalista, la luz LED se puede colocar en cualquier lugar, como una mesita de noche, una estantería, una mesa, una mesa de comedor, etc
-- INALÁMBRICO Y RECARGABLE: la lámpara de mesa inalámbrica tiene una batería recargable de 1800 mAh incorporada
-- 3 COLORES: esta lámpara de mesa tiene 3 colores de iluminación: luz blanca, blanca cálida, luz , puede seleccionar usar según las necesidades, presione prolongadamente para atenuación continua
-- La lámpara de mesa adopta una carcasa de metal, una pantalla de acrílico transparente, un proceso de galvanoplastia superficial y un diseño de base antideslizante, resistente y estable
-- Diseño elegante: construido con una carcasa de metal resistente y una pantalla acrílica transparente, esta lámpara combina durabilidad con elegancia</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>Decoración y hogar</t>
-        </is>
-      </c>
-      <c r="E86" t="n">
-        <v>35000</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>BANDEJA 3 NIVELES ACRÍLICO DORADO TORRE POSTRES CUPCAKES DULCES APERITIVOS DESMONTABLE ELEGANTE PLATEADO TCP311</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>TCP311</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>- Ideal para fiestas, bodas, cumpleaños, baby showers, eventos corporativos o incluso para la decoración del hogar, este soporte es perfecto para exhibir dulces gourmet, cupcakes, minitartas, frutas, aperitivos salados o pequeños obsequios
-- Su diseño sofisticado aporta un toque de lujo a la mesa, mientras que el material acrílico de alta calidad garantiza que sea ligero, duradero y fácil de limpiar
-- Gracias a su estructura robusta y acabado en tono dorado, combina a la perfección con diversos estilos de decoración, desde el clásico hasta el moderno
-- Material: Acrílico resistente
-- Color: Transparente con detalles dorados</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>Decoración y hogar</t>
-        </is>
-      </c>
-      <c r="E87" t="n">
-        <v>45000</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>BANDEJA 3 NIVELES ACRÍLICO DORADO TORRE POSTRES CUPCAKES DULCES APERITIVOS DESMONTABLE ELEGANTE DORADO TCP311D</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>TCP311D</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>- Ideal para fiestas, bodas, cumpleaños, baby showers, eventos corporativos o incluso para la decoración del hogar, este soporte es perfecto para exhibir dulces gourmet, cupcakes, minitartas, frutas, aperitivos salados o pequeños obsequios
-- Su diseño sofisticado aporta un toque de lujo a la mesa, mientras que el material acrílico de alta calidad garantiza que sea ligero, duradero y fácil de limpiar
-- Gracias a su estructura robusta y acabado en tono dorado, combina a la perfección con diversos estilos de decoración, desde el clásico hasta el moderno
-- Material: Acrílico resistente
-- Color: Transparente con detalles dorados</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>Decoración y hogar</t>
-        </is>
-      </c>
-      <c r="E88" t="n">
-        <v>45000</v>
       </c>
     </row>
   </sheetData>
@@ -3519,6 +3181,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="26.1" customHeight="1" s="25">
       <c r="A3" s="28" t="inlineStr">
         <is>
@@ -3690,6 +3353,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25" ht="26.1" customHeight="1" s="25">
       <c r="A25" s="28" t="inlineStr">
         <is>

</xml_diff>